<commit_message>
chore(audit): review b929281, record 83 findings, MFA policy and release gates
</commit_message>
<xml_diff>
--- a/audits/FORTLESS_MASTER_SECURITY_UI_BUG_TRACKER.xlsx
+++ b/audits/FORTLESS_MASTER_SECURITY_UI_BUG_TRACKER.xlsx
@@ -2,13 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Findings" sheetId="1" r:id="Ra3a5dbe249104833"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="R90d3d1708bb74a7a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit Coverage" sheetId="3" r:id="Rdfc7644eca3241cf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Push History" sheetId="4" r:id="Rc3759e6a874b4c5a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status History" sheetId="5" r:id="R1d4e5e9505da4b79"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ideas Separate" sheetId="6" r:id="R489c39e9a29c434c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How To Update" sheetId="7" r:id="Rd50d91fb8c79463d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Findings" sheetId="1" r:id="R1d6ec6185841420d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="Rc951f5f95f5f4319"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit Coverage" sheetId="3" r:id="R47ae13c680fa4d4c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Push History" sheetId="4" r:id="R1f137a69bd2f4a61"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status History" sheetId="5" r:id="R151a16a584ca4237"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ideas Separate" sheetId="6" r:id="R6c7e1f089c3045b1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How To Update" sheetId="7" r:id="R7acc59c623d84553"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MFA Policy" sheetId="8" r:id="R66035a945ea541ab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="9" r:id="R20d1a623fa8a4960"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -19,7 +21,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="15">
+  <x:fonts count="16">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -104,8 +106,14 @@
       <x:color rgb="FFFFFFFF"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="14"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="11">
+  <x:fills count="13">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -157,6 +165,16 @@
         <x:fgColor rgb="FFF8FAFD"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF142235"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1D4254"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="2">
     <x:border/>
@@ -165,7 +183,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="73">
+  <x:cellXfs count="77">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -287,6 +305,10 @@
     <x:xf numFmtId="0" fontId="14" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="14" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="15" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -350,35 +372,35 @@
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF1D6"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF3E8FF"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDBEAFE"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE0F7E9"/>
         </x:patternFill>
       </x:fill>
@@ -668,7 +690,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>MASTER TRACKER  •  6203687 HEAD rechecked 19 Oct 2026  •  11 added findings  •  fixes still require independent tests</x:v>
+        <x:v>MASTER TRACKER  •  b929281 rechecked 19 Oct 2026  •  9 new defects; production validation still pending</x:v>
       </x:c>
       <x:c r="B2" s="7"/>
       <x:c r="C2" s="7"/>
@@ -934,7 +956,7 @@
         <x:v>Pending MFA challenges have an overly long lifetime and per-session attempt accounting</x:v>
       </x:c>
       <x:c r="F7" s="18" t="str">
-        <x:v>PARTIAL</x:v>
+        <x:v>FIXED_IN_CODE</x:v>
       </x:c>
       <x:c r="G7" s="18" t="str">
         <x:v>2026-10-19</x:v>
@@ -943,10 +965,10 @@
         <x:v>2026-10-19</x:v>
       </x:c>
       <x:c r="I7" s="18" t="str">
-        <x:v>9dacfcb</x:v>
+        <x:v>b929281</x:v>
       </x:c>
       <x:c r="J7" s="18" t="str">
-        <x:v>6203687</x:v>
+        <x:v>b929281</x:v>
       </x:c>
       <x:c r="K7" s="18" t="str"/>
       <x:c r="L7" s="18" t="str">
@@ -969,7 +991,7 @@
         <x:v>Coding AI</x:v>
       </x:c>
       <x:c r="S7" s="18" t="str">
-        <x:v>Pending MFA 15-min limit added; per-user attempt reset issue remains FTL-SEC-202</x:v>
+        <x:v>Pending MFA 15-min limit added; per-user attempt reset issue remains FTL-SEC-202 | b929281: Pending-MFA 15-min TTL and account-wide failures in auth.ts; requires runtime test.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="66" customHeight="1">
@@ -1668,7 +1690,7 @@
         <x:v>Existing TOTP can be silently replaced with an unconfirmed factor</x:v>
       </x:c>
       <x:c r="F21" s="18" t="str">
-        <x:v>OPEN</x:v>
+        <x:v>FIXED_IN_CODE</x:v>
       </x:c>
       <x:c r="G21" s="18" t="str">
         <x:v>2026-10-19</x:v>
@@ -1677,10 +1699,10 @@
         <x:v>2026-10-19</x:v>
       </x:c>
       <x:c r="I21" s="18" t="str">
-        <x:v>6203687</x:v>
+        <x:v>b929281</x:v>
       </x:c>
       <x:c r="J21" s="18" t="str">
-        <x:v>6203687</x:v>
+        <x:v>b929281</x:v>
       </x:c>
       <x:c r="K21" s="18" t="str">
         <x:v>src/modules/identity/auth.ts, src/server.ts</x:v>
@@ -1706,7 +1728,9 @@
       <x:c r="R21" s="18" t="str">
         <x:v>Coding AI</x:v>
       </x:c>
-      <x:c r="S21" s="18" t="str"/>
+      <x:c r="S21" s="18" t="str">
+        <x:v>| b929281: Confirmed factor remains active; pending_secret_encrypted used for replacement.</x:v>
+      </x:c>
     </x:row>
     <x:row r="22" ht="66" customHeight="1">
       <x:c r="A22" s="18" t="str">
@@ -1725,7 +1749,7 @@
         <x:v>Global MFA attempt limit resets on same-device relogin</x:v>
       </x:c>
       <x:c r="F22" s="18" t="str">
-        <x:v>OPEN</x:v>
+        <x:v>FIXED_IN_CODE</x:v>
       </x:c>
       <x:c r="G22" s="18" t="str">
         <x:v>2026-10-19</x:v>
@@ -1734,10 +1758,10 @@
         <x:v>2026-10-19</x:v>
       </x:c>
       <x:c r="I22" s="18" t="str">
-        <x:v>6203687</x:v>
+        <x:v>b929281</x:v>
       </x:c>
       <x:c r="J22" s="18" t="str">
-        <x:v>6203687</x:v>
+        <x:v>b929281</x:v>
       </x:c>
       <x:c r="K22" s="18" t="str">
         <x:v>src/modules/identity/auth.ts</x:v>
@@ -1763,7 +1787,9 @@
       <x:c r="R22" s="18" t="str">
         <x:v>Coding AI</x:v>
       </x:c>
-      <x:c r="S22" s="18" t="str"/>
+      <x:c r="S22" s="18" t="str">
+        <x:v>| b929281: MFA failures now queried by user_id across all pending sessions.</x:v>
+      </x:c>
     </x:row>
     <x:row r="23" ht="66" customHeight="1">
       <x:c r="A23" s="18" t="str">
@@ -1782,7 +1808,7 @@
         <x:v>Recovery-code regeneration lacks sensitive-action reauthentication</x:v>
       </x:c>
       <x:c r="F23" s="18" t="str">
-        <x:v>OPEN</x:v>
+        <x:v>FIXED_IN_CODE</x:v>
       </x:c>
       <x:c r="G23" s="18" t="str">
         <x:v>2026-10-19</x:v>
@@ -1791,10 +1817,10 @@
         <x:v>2026-10-19</x:v>
       </x:c>
       <x:c r="I23" s="18" t="str">
-        <x:v>6203687</x:v>
+        <x:v>b929281</x:v>
       </x:c>
       <x:c r="J23" s="18" t="str">
-        <x:v>6203687</x:v>
+        <x:v>b929281</x:v>
       </x:c>
       <x:c r="K23" s="18" t="str">
         <x:v>src/server.ts, src/modules/identity/auth.ts</x:v>
@@ -1820,7 +1846,9 @@
       <x:c r="R23" s="18" t="str">
         <x:v>Coding AI</x:v>
       </x:c>
-      <x:c r="S23" s="18" t="str"/>
+      <x:c r="S23" s="18" t="str">
+        <x:v>| b929281: Recovery-code regeneration protected by requireRecentStepUp.</x:v>
+      </x:c>
     </x:row>
     <x:row r="24" ht="66" customHeight="1">
       <x:c r="A24" s="18" t="str">
@@ -1839,7 +1867,7 @@
         <x:v>Monthly Stripe plan for nonmonthly quote intervals</x:v>
       </x:c>
       <x:c r="F24" s="18" t="str">
-        <x:v>OPEN</x:v>
+        <x:v>PARTIAL</x:v>
       </x:c>
       <x:c r="G24" s="18" t="str">
         <x:v>2026-10-19</x:v>
@@ -1848,10 +1876,10 @@
         <x:v>2026-10-19</x:v>
       </x:c>
       <x:c r="I24" s="18" t="str">
-        <x:v>6203687</x:v>
+        <x:v>b929281</x:v>
       </x:c>
       <x:c r="J24" s="18" t="str">
-        <x:v>6203687</x:v>
+        <x:v>b929281</x:v>
       </x:c>
       <x:c r="K24" s="18" t="str">
         <x:v>src/modules/pricing/quote.ts, src/modules/checkout/checkout.ts</x:v>
@@ -1877,7 +1905,9 @@
       <x:c r="R24" s="18" t="str">
         <x:v>Coding AI</x:v>
       </x:c>
-      <x:c r="S24" s="18" t="str"/>
+      <x:c r="S24" s="18" t="str">
+        <x:v>| b929281: Stripe recurring interval mapped correctly; webhook still persists local subscriptions as MONTHLY.</x:v>
+      </x:c>
     </x:row>
     <x:row r="25" ht="66" customHeight="1">
       <x:c r="A25" s="18" t="str">
@@ -1896,7 +1926,7 @@
         <x:v>Refund/chargeback changes local service state without provider action</x:v>
       </x:c>
       <x:c r="F25" s="18" t="str">
-        <x:v>OPEN</x:v>
+        <x:v>PARTIAL</x:v>
       </x:c>
       <x:c r="G25" s="18" t="str">
         <x:v>2026-10-19</x:v>
@@ -1905,10 +1935,10 @@
         <x:v>2026-10-19</x:v>
       </x:c>
       <x:c r="I25" s="18" t="str">
-        <x:v>6203687</x:v>
+        <x:v>b929281</x:v>
       </x:c>
       <x:c r="J25" s="18" t="str">
-        <x:v>6203687</x:v>
+        <x:v>b929281</x:v>
       </x:c>
       <x:c r="K25" s="18" t="str">
         <x:v>src/modules/payments/webhooks.ts</x:v>
@@ -1934,7 +1964,9 @@
       <x:c r="R25" s="18" t="str">
         <x:v>Coding AI</x:v>
       </x:c>
-      <x:c r="S25" s="18" t="str"/>
+      <x:c r="S25" s="18" t="str">
+        <x:v>| b929281: Refund/dispute webhook enqueues suspend/terminate actions; staff refund path still bypasses PSP/provider.</x:v>
+      </x:c>
     </x:row>
     <x:row r="26" ht="66" customHeight="1">
       <x:c r="A26" s="18" t="str">
@@ -1953,7 +1985,7 @@
         <x:v>Distinct Stripe events for same payment can re-run fulfillment</x:v>
       </x:c>
       <x:c r="F26" s="18" t="str">
-        <x:v>OPEN</x:v>
+        <x:v>FIXED_IN_CODE</x:v>
       </x:c>
       <x:c r="G26" s="18" t="str">
         <x:v>2026-10-19</x:v>
@@ -1962,10 +1994,10 @@
         <x:v>2026-10-19</x:v>
       </x:c>
       <x:c r="I26" s="18" t="str">
-        <x:v>6203687</x:v>
+        <x:v>b929281</x:v>
       </x:c>
       <x:c r="J26" s="18" t="str">
-        <x:v>6203687</x:v>
+        <x:v>b929281</x:v>
       </x:c>
       <x:c r="K26" s="18" t="str">
         <x:v>src/modules/payments/webhooks.ts, src/database/schema.ts</x:v>
@@ -1991,7 +2023,9 @@
       <x:c r="R26" s="18" t="str">
         <x:v>Coding AI</x:v>
       </x:c>
-      <x:c r="S26" s="18" t="str"/>
+      <x:c r="S26" s="18" t="str">
+        <x:v>| b929281: Webhook checks payment_attempts.status/order.status before repeated fulfillment.</x:v>
+      </x:c>
     </x:row>
     <x:row r="27" ht="66" customHeight="1">
       <x:c r="A27" s="18" t="str">
@@ -2010,7 +2044,7 @@
         <x:v>Stripe PaymentIntent/refund/dispute correlation does not use actual Stripe IDs</x:v>
       </x:c>
       <x:c r="F27" s="18" t="str">
-        <x:v>OPEN</x:v>
+        <x:v>PARTIAL</x:v>
       </x:c>
       <x:c r="G27" s="18" t="str">
         <x:v>2026-10-19</x:v>
@@ -2019,10 +2053,10 @@
         <x:v>2026-10-19</x:v>
       </x:c>
       <x:c r="I27" s="18" t="str">
-        <x:v>6203687</x:v>
+        <x:v>b929281</x:v>
       </x:c>
       <x:c r="J27" s="18" t="str">
-        <x:v>6203687</x:v>
+        <x:v>b929281</x:v>
       </x:c>
       <x:c r="K27" s="18" t="str">
         <x:v>src/modules/checkout/checkout.ts, src/modules/payments/webhooks.ts, src/database/schema.ts</x:v>
@@ -2048,7 +2082,9 @@
       <x:c r="R27" s="18" t="str">
         <x:v>Coding AI</x:v>
       </x:c>
-      <x:c r="S27" s="18" t="str"/>
+      <x:c r="S27" s="18" t="str">
+        <x:v>| b929281: Real payment_intent IDs stored; invoice.paid settlement scopes invoices by account, not Stripe invoice.</x:v>
+      </x:c>
     </x:row>
     <x:row r="28" ht="66" customHeight="1">
       <x:c r="A28" s="18" t="str">
@@ -2067,7 +2103,7 @@
         <x:v>Subscription renewal flow not aligned with Stripe's auto-renewal</x:v>
       </x:c>
       <x:c r="F28" s="18" t="str">
-        <x:v>OPEN</x:v>
+        <x:v>PARTIAL</x:v>
       </x:c>
       <x:c r="G28" s="18" t="str">
         <x:v>2026-10-19</x:v>
@@ -2076,10 +2112,10 @@
         <x:v>2026-10-19</x:v>
       </x:c>
       <x:c r="I28" s="18" t="str">
-        <x:v>6203687</x:v>
+        <x:v>b929281</x:v>
       </x:c>
       <x:c r="J28" s="18" t="str">
-        <x:v>6203687</x:v>
+        <x:v>b929281</x:v>
       </x:c>
       <x:c r="K28" s="18" t="str">
         <x:v>src/modules/billing/renewal-dunning.ts, src/modules/payments/webhooks.ts</x:v>
@@ -2105,7 +2141,9 @@
       <x:c r="R28" s="18" t="str">
         <x:v>Coding AI</x:v>
       </x:c>
-      <x:c r="S28" s="18" t="str"/>
+      <x:c r="S28" s="18" t="str">
+        <x:v>| b929281: Stripe subscriptions exempted from local dunning; invoice.paid wrongly settles all account invoices.</x:v>
+      </x:c>
     </x:row>
     <x:row r="29" ht="66" customHeight="1">
       <x:c r="A29" s="18" t="str">
@@ -2181,7 +2219,7 @@
         <x:v>Worker uses one global provider for all service types</x:v>
       </x:c>
       <x:c r="F30" s="18" t="str">
-        <x:v>OPEN</x:v>
+        <x:v>PARTIAL</x:v>
       </x:c>
       <x:c r="G30" s="18" t="str">
         <x:v>2026-10-19</x:v>
@@ -2190,10 +2228,10 @@
         <x:v>2026-10-19</x:v>
       </x:c>
       <x:c r="I30" s="18" t="str">
-        <x:v>6203687</x:v>
+        <x:v>b929281</x:v>
       </x:c>
       <x:c r="J30" s="18" t="str">
-        <x:v>6203687</x:v>
+        <x:v>b929281</x:v>
       </x:c>
       <x:c r="K30" s="18" t="str">
         <x:v>src/modules/outbox/worker.ts, src/modules/checkout/checkout.ts, src/modules/payments/webhooks.ts</x:v>
@@ -2219,7 +2257,9 @@
       <x:c r="R30" s="18" t="str">
         <x:v>Coding AI</x:v>
       </x:c>
-      <x:c r="S30" s="18" t="str"/>
+      <x:c r="S30" s="18" t="str">
+        <x:v>| b929281: Dispatch by provider_type added, but CPANEL/VPS dispatch still constructs mock adapters in worker.</x:v>
+      </x:c>
     </x:row>
     <x:row r="31" ht="66" customHeight="1">
       <x:c r="A31" s="18" t="str">
@@ -2238,7 +2278,7 @@
         <x:v>Hardcoded node fallback and no capacity-aware assignment on paid/free checkout</x:v>
       </x:c>
       <x:c r="F31" s="18" t="str">
-        <x:v>OPEN</x:v>
+        <x:v>PARTIAL</x:v>
       </x:c>
       <x:c r="G31" s="18" t="str">
         <x:v>2026-10-19</x:v>
@@ -2247,10 +2287,10 @@
         <x:v>2026-10-19</x:v>
       </x:c>
       <x:c r="I31" s="18" t="str">
-        <x:v>6203687</x:v>
+        <x:v>b929281</x:v>
       </x:c>
       <x:c r="J31" s="18" t="str">
-        <x:v>6203687</x:v>
+        <x:v>b929281</x:v>
       </x:c>
       <x:c r="K31" s="18" t="str">
         <x:v>src/modules/checkout/checkout.ts, src/modules/payments/webhooks.ts</x:v>
@@ -2276,7 +2316,9 @@
       <x:c r="R31" s="18" t="str">
         <x:v>Coding AI</x:v>
       </x:c>
-      <x:c r="S31" s="18" t="str"/>
+      <x:c r="S31" s="18" t="str">
+        <x:v>| b929281: Hardcoded node_fra_01 removed; fallback still chooses wrong region/no-capacity nodes.</x:v>
+      </x:c>
     </x:row>
     <x:row r="32" ht="66" customHeight="1">
       <x:c r="A32" s="18" t="str">
@@ -2295,7 +2337,7 @@
         <x:v>Capacity concurrency check is not atomic with reservation/update</x:v>
       </x:c>
       <x:c r="F32" s="18" t="str">
-        <x:v>OPEN</x:v>
+        <x:v>FIXED_IN_CODE</x:v>
       </x:c>
       <x:c r="G32" s="18" t="str">
         <x:v>2026-10-19</x:v>
@@ -2304,10 +2346,10 @@
         <x:v>2026-10-19</x:v>
       </x:c>
       <x:c r="I32" s="18" t="str">
-        <x:v>6203687</x:v>
+        <x:v>b929281</x:v>
       </x:c>
       <x:c r="J32" s="18" t="str">
-        <x:v>6203687</x:v>
+        <x:v>b929281</x:v>
       </x:c>
       <x:c r="K32" s="18" t="str">
         <x:v>src/modules/outbox/worker.ts</x:v>
@@ -2333,7 +2375,9 @@
       <x:c r="R32" s="18" t="str">
         <x:v>Coding AI</x:v>
       </x:c>
-      <x:c r="S32" s="18" t="str"/>
+      <x:c r="S32" s="18" t="str">
+        <x:v>| b929281: Worker now atomically reserves capacity with conditional UPDATE.</x:v>
+      </x:c>
     </x:row>
     <x:row r="33" ht="66" customHeight="1">
       <x:c r="A33" s="18" t="str">
@@ -2409,7 +2453,7 @@
         <x:v>Domain search is not external registrar availability</x:v>
       </x:c>
       <x:c r="F34" s="18" t="str">
-        <x:v>OPEN</x:v>
+        <x:v>PARTIAL</x:v>
       </x:c>
       <x:c r="G34" s="18" t="str">
         <x:v>2026-10-19</x:v>
@@ -2418,10 +2462,10 @@
         <x:v>2026-10-19</x:v>
       </x:c>
       <x:c r="I34" s="18" t="str">
-        <x:v>6203687</x:v>
+        <x:v>b929281</x:v>
       </x:c>
       <x:c r="J34" s="18" t="str">
-        <x:v>6203687</x:v>
+        <x:v>b929281</x:v>
       </x:c>
       <x:c r="K34" s="18" t="str">
         <x:v>src/modules/domains/dns.ts</x:v>
@@ -2445,7 +2489,9 @@
       <x:c r="R34" s="18" t="str">
         <x:v>Coding AI</x:v>
       </x:c>
-      <x:c r="S34" s="18" t="str"/>
+      <x:c r="S34" s="18" t="str">
+        <x:v>| b929281: Search discloses LOCAL_ZONE_AVAILABLE, but still returns available:true without registrar check.</x:v>
+      </x:c>
     </x:row>
     <x:row r="35" ht="66" customHeight="1">
       <x:c r="A35" s="18" t="str">
@@ -2464,7 +2510,7 @@
         <x:v>Locally created zone advertised ACTIVE without DNS authority proof</x:v>
       </x:c>
       <x:c r="F35" s="18" t="str">
-        <x:v>OPEN</x:v>
+        <x:v>PARTIAL</x:v>
       </x:c>
       <x:c r="G35" s="18" t="str">
         <x:v>2026-10-19</x:v>
@@ -2473,10 +2519,10 @@
         <x:v>2026-10-19</x:v>
       </x:c>
       <x:c r="I35" s="18" t="str">
-        <x:v>6203687</x:v>
+        <x:v>b929281</x:v>
       </x:c>
       <x:c r="J35" s="18" t="str">
-        <x:v>6203687</x:v>
+        <x:v>b929281</x:v>
       </x:c>
       <x:c r="K35" s="18" t="str">
         <x:v>src/modules/domains/dns.ts</x:v>
@@ -2502,7 +2548,9 @@
       <x:c r="R35" s="18" t="str">
         <x:v>Coding AI</x:v>
       </x:c>
-      <x:c r="S35" s="18" t="str"/>
+      <x:c r="S35" s="18" t="str">
+        <x:v>| b929281: Zone has pending/delegation distinction; authoritative DNS/registrar integration not verified.</x:v>
+      </x:c>
     </x:row>
     <x:row r="36" ht="66" customHeight="1">
       <x:c r="A36" s="18" t="str">
@@ -2521,7 +2569,7 @@
         <x:v>Recovery-code entropy only ~32 bits, fast hash</x:v>
       </x:c>
       <x:c r="F36" s="18" t="str">
-        <x:v>OPEN</x:v>
+        <x:v>FIXED_IN_CODE</x:v>
       </x:c>
       <x:c r="G36" s="18" t="str">
         <x:v>2026-10-19</x:v>
@@ -2530,10 +2578,10 @@
         <x:v>2026-10-19</x:v>
       </x:c>
       <x:c r="I36" s="18" t="str">
-        <x:v>6203687</x:v>
+        <x:v>b929281</x:v>
       </x:c>
       <x:c r="J36" s="18" t="str">
-        <x:v>6203687</x:v>
+        <x:v>b929281</x:v>
       </x:c>
       <x:c r="K36" s="18" t="str">
         <x:v>src/modules/identity/auth.ts</x:v>
@@ -2559,7 +2607,9 @@
       <x:c r="R36" s="18" t="str">
         <x:v>Coding AI</x:v>
       </x:c>
-      <x:c r="S36" s="18" t="str"/>
+      <x:c r="S36" s="18" t="str">
+        <x:v>| b929281: Recovery codes now 128-bit generated from randomBytes(16).</x:v>
+      </x:c>
     </x:row>
     <x:row r="37" ht="66" customHeight="1">
       <x:c r="A37" s="18" t="str">
@@ -2578,7 +2628,7 @@
         <x:v>Account-and-IP login throttle has no account-wide distributed limit</x:v>
       </x:c>
       <x:c r="F37" s="18" t="str">
-        <x:v>OPEN</x:v>
+        <x:v>FIXED_IN_CODE</x:v>
       </x:c>
       <x:c r="G37" s="18" t="str">
         <x:v>2026-10-19</x:v>
@@ -2587,10 +2637,10 @@
         <x:v>2026-10-19</x:v>
       </x:c>
       <x:c r="I37" s="18" t="str">
-        <x:v>6203687</x:v>
+        <x:v>b929281</x:v>
       </x:c>
       <x:c r="J37" s="18" t="str">
-        <x:v>6203687</x:v>
+        <x:v>b929281</x:v>
       </x:c>
       <x:c r="K37" s="18" t="str">
         <x:v>src/modules/identity/auth.ts</x:v>
@@ -2614,7 +2664,9 @@
       <x:c r="R37" s="18" t="str">
         <x:v>Coding AI</x:v>
       </x:c>
-      <x:c r="S37" s="18" t="str"/>
+      <x:c r="S37" s="18" t="str">
+        <x:v>| b929281: isLoginThrottled now counts 10 failures account-wide independent of IP.</x:v>
+      </x:c>
     </x:row>
     <x:row r="38" ht="66" customHeight="1">
       <x:c r="A38" s="18" t="str">
@@ -2633,7 +2685,7 @@
         <x:v>Billing-only workspace user sees server power buttons</x:v>
       </x:c>
       <x:c r="F38" s="18" t="str">
-        <x:v>OPEN</x:v>
+        <x:v>FIXED_IN_CODE</x:v>
       </x:c>
       <x:c r="G38" s="18" t="str">
         <x:v>2026-10-19</x:v>
@@ -2642,10 +2694,10 @@
         <x:v>2026-10-19</x:v>
       </x:c>
       <x:c r="I38" s="18" t="str">
-        <x:v>6203687</x:v>
+        <x:v>b929281</x:v>
       </x:c>
       <x:c r="J38" s="18" t="str">
-        <x:v>6203687</x:v>
+        <x:v>b929281</x:v>
       </x:c>
       <x:c r="K38" s="18" t="str">
         <x:v>src/frontend/client/pages/dashboard/index.ts, src/modules/provisioning/service-access.ts</x:v>
@@ -2669,7 +2721,9 @@
       <x:c r="R38" s="18" t="str">
         <x:v>Coding AI</x:v>
       </x:c>
-      <x:c r="S38" s="18" t="str"/>
+      <x:c r="S38" s="18" t="str">
+        <x:v>| b929281: Service list checks user_can_control, detailed page checks explicit permissions; runtime E2E needed.</x:v>
+      </x:c>
     </x:row>
     <x:row r="39" ht="66" customHeight="1">
       <x:c r="A39" s="18" t="str">
@@ -2688,7 +2742,7 @@
         <x:v>Service detail renders Pterodactyl actions for incompatible provider types</x:v>
       </x:c>
       <x:c r="F39" s="18" t="str">
-        <x:v>OPEN</x:v>
+        <x:v>FIXED_IN_CODE</x:v>
       </x:c>
       <x:c r="G39" s="18" t="str">
         <x:v>2026-10-19</x:v>
@@ -2697,10 +2751,10 @@
         <x:v>2026-10-19</x:v>
       </x:c>
       <x:c r="I39" s="18" t="str">
-        <x:v>6203687</x:v>
+        <x:v>b929281</x:v>
       </x:c>
       <x:c r="J39" s="18" t="str">
-        <x:v>6203687</x:v>
+        <x:v>b929281</x:v>
       </x:c>
       <x:c r="K39" s="18" t="str">
         <x:v>src/frontend/client/pages/services/index.ts</x:v>
@@ -2724,7 +2778,9 @@
       <x:c r="R39" s="18" t="str">
         <x:v>Coding AI</x:v>
       </x:c>
-      <x:c r="S39" s="18" t="str"/>
+      <x:c r="S39" s="18" t="str">
+        <x:v>| b929281: Service details filter provider tabs by capabilities and permissions.</x:v>
+      </x:c>
     </x:row>
     <x:row r="40" ht="66" customHeight="1">
       <x:c r="A40" s="18" t="str">
@@ -2743,7 +2799,7 @@
         <x:v>Route navigation is not race-safe for async page loaders</x:v>
       </x:c>
       <x:c r="F40" s="18" t="str">
-        <x:v>OPEN</x:v>
+        <x:v>PARTIAL</x:v>
       </x:c>
       <x:c r="G40" s="18" t="str">
         <x:v>2026-10-19</x:v>
@@ -2752,10 +2808,10 @@
         <x:v>2026-10-19</x:v>
       </x:c>
       <x:c r="I40" s="18" t="str">
-        <x:v>6203687</x:v>
+        <x:v>b929281</x:v>
       </x:c>
       <x:c r="J40" s="18" t="str">
-        <x:v>6203687</x:v>
+        <x:v>b929281</x:v>
       </x:c>
       <x:c r="K40" s="18" t="str">
         <x:v>src/frontend/core/router/router.ts</x:v>
@@ -2781,7 +2837,9 @@
       <x:c r="R40" s="18" t="str">
         <x:v>Coding AI</x:v>
       </x:c>
-      <x:c r="S40" s="18" t="str"/>
+      <x:c r="S40" s="18" t="str">
+        <x:v>| b929281: Router has sequence and AbortController; async page fetches do not consistently use signal guard.</x:v>
+      </x:c>
     </x:row>
     <x:row r="41" ht="66" customHeight="1">
       <x:c r="A41" s="18" t="str">
@@ -2800,7 +2858,7 @@
         <x:v>Canonical visual QA checks 22 routes, omits 2 required views</x:v>
       </x:c>
       <x:c r="F41" s="18" t="str">
-        <x:v>OPEN</x:v>
+        <x:v>PARTIAL</x:v>
       </x:c>
       <x:c r="G41" s="18" t="str">
         <x:v>2026-10-19</x:v>
@@ -2809,10 +2867,10 @@
         <x:v>2026-10-19</x:v>
       </x:c>
       <x:c r="I41" s="18" t="str">
-        <x:v>6203687</x:v>
+        <x:v>b929281</x:v>
       </x:c>
       <x:c r="J41" s="18" t="str">
-        <x:v>6203687</x:v>
+        <x:v>b929281</x:v>
       </x:c>
       <x:c r="K41" s="18" t="str">
         <x:v>scripts/verify-views.py</x:v>
@@ -2837,7 +2895,7 @@
         <x:v>Coding AI</x:v>
       </x:c>
       <x:c r="S41" s="18" t="str">
-        <x:v>22/24 routes covered by screenshot script, incomplete visual parity checks</x:v>
+        <x:v>22/24 routes covered by screenshot script, incomplete visual parity checks | b929281: 24 route definitions present in verify-views.py, but no authenticated fixture/pixel reference comparison.</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="66" customHeight="1">
@@ -2866,10 +2924,10 @@
         <x:v>2026-10-19</x:v>
       </x:c>
       <x:c r="I42" s="18" t="str">
-        <x:v>6203687</x:v>
+        <x:v>b929281</x:v>
       </x:c>
       <x:c r="J42" s="18" t="str">
-        <x:v>6203687</x:v>
+        <x:v>b929281</x:v>
       </x:c>
       <x:c r="K42" s="18" t="str">
         <x:v>src/frontend/client/pages/dashboard/index.ts</x:v>
@@ -2893,7 +2951,9 @@
       <x:c r="R42" s="18" t="str">
         <x:v>Coding AI</x:v>
       </x:c>
-      <x:c r="S42" s="18" t="str"/>
+      <x:c r="S42" s="18" t="str">
+        <x:v>| b929281: Refresh renderServices catches API error internally, then caller still fires refreshed toast.</x:v>
+      </x:c>
     </x:row>
     <x:row r="43" ht="66" customHeight="1">
       <x:c r="A43" s="18" t="str">
@@ -2912,7 +2972,7 @@
         <x:v>Client power controls do not use runtime-action eligibility or live provider-specific state comprehensively</x:v>
       </x:c>
       <x:c r="F43" s="18" t="str">
-        <x:v>OPEN</x:v>
+        <x:v>PARTIAL</x:v>
       </x:c>
       <x:c r="G43" s="18" t="str">
         <x:v>2026-10-19</x:v>
@@ -2921,10 +2981,10 @@
         <x:v>2026-10-19</x:v>
       </x:c>
       <x:c r="I43" s="18" t="str">
-        <x:v>6203687</x:v>
+        <x:v>b929281</x:v>
       </x:c>
       <x:c r="J43" s="18" t="str">
-        <x:v>6203687</x:v>
+        <x:v>b929281</x:v>
       </x:c>
       <x:c r="K43" s="18" t="str">
         <x:v>src/frontend/client/pages/services/status.ts, src/frontend/client/pages/dashboard/index.ts, src/frontend/client/pages/services/index.ts</x:v>
@@ -2948,7 +3008,9 @@
       <x:c r="R43" s="18" t="str">
         <x:v>Coding AI</x:v>
       </x:c>
-      <x:c r="S43" s="18" t="str"/>
+      <x:c r="S43" s="18" t="str">
+        <x:v>| b929281: Buttons account for contract/runtime status but per-button action permission and provider feedback remain incomplete.</x:v>
+      </x:c>
     </x:row>
     <x:row r="44" ht="66" customHeight="1">
       <x:c r="A44" s="18" t="str">
@@ -4934,6 +4996,537 @@
       </x:c>
       <x:c r="S77" s="18" t="str">
         <x:v>UX inconsistency, not authorization bypass; protected route correctly denies navigation.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="78" ht="50" customHeight="1">
+      <x:c r="A78" s="66" t="str">
+        <x:v>NEW-330</x:v>
+      </x:c>
+      <x:c r="B78" s="66" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C78" s="66" t="str">
+        <x:v>CRITICAL</x:v>
+      </x:c>
+      <x:c r="D78" s="66" t="str">
+        <x:v>Billing</x:v>
+      </x:c>
+      <x:c r="E78" s="66" t="str">
+        <x:v>Stripe invoice.paid can mark unrelated issued invoices paid</x:v>
+      </x:c>
+      <x:c r="F78" s="66" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="G78" s="66" t="str">
+        <x:v>2026-10-19</x:v>
+      </x:c>
+      <x:c r="H78" s="66" t="str">
+        <x:v>2026-10-19</x:v>
+      </x:c>
+      <x:c r="I78" s="66" t="str">
+        <x:v>b929281</x:v>
+      </x:c>
+      <x:c r="J78" s="66" t="str">
+        <x:v>b929281</x:v>
+      </x:c>
+      <x:c r="K78" s="66" t="str">
+        <x:v>src/modules/payments/webhooks.ts:218-245</x:v>
+      </x:c>
+      <x:c r="L78" s="66" t="str">
+        <x:v>invoice.paid resolves a subscription, then UPDATE invoices SET status='PAID' WHERE account_id=? AND status='ISSUED'; no Stripe invoice ID or amount is joined.</x:v>
+      </x:c>
+      <x:c r="M78" s="66" t="str">
+        <x:v>One successful renewal may falsely settle every other open issued invoice for that account.</x:v>
+      </x:c>
+      <x:c r="N78" s="66" t="str">
+        <x:v>Persist and uniquely map Stripe invoice ID and payment to ONE Fortless invoice/subscription; validate money/currency and idempotence, never bulk-settle by account.</x:v>
+      </x:c>
+      <x:c r="O78" s="66" t="str">
+        <x:v>Create 2 active subscriptions plus 3 issued invoices for same account; paying only one must update exactly its matching invoice.</x:v>
+      </x:c>
+      <x:c r="P78" s="66" t="str">
+        <x:v>FORTLESS_AUDIT_BOUNTY_b929281.md</x:v>
+      </x:c>
+      <x:c r="Q78" s="66" t="str">
+        <x:v>https://github.com/trencito42/fortless/blob/b9292811a22159a28a7159deee2c7ff27f41a873/src/modules/payments/webhooks.ts</x:v>
+      </x:c>
+      <x:c r="R78" s="66" t="str">
+        <x:v>Coding AI</x:v>
+      </x:c>
+      <x:c r="S78" s="66" t="str">
+        <x:v>New code finding; verified statically, no authorized runtime exploit or E2E validation.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="79" ht="50" customHeight="1">
+      <x:c r="A79" s="66" t="str">
+        <x:v>NEW-331</x:v>
+      </x:c>
+      <x:c r="B79" s="66" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C79" s="66" t="str">
+        <x:v>HIGH</x:v>
+      </x:c>
+      <x:c r="D79" s="66" t="str">
+        <x:v>Authorization</x:v>
+      </x:c>
+      <x:c r="E79" s="66" t="str">
+        <x:v>TECH_ADMIN can invite a new workspace OWNER</x:v>
+      </x:c>
+      <x:c r="F79" s="66" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="G79" s="66" t="str">
+        <x:v>2026-10-19</x:v>
+      </x:c>
+      <x:c r="H79" s="66" t="str">
+        <x:v>2026-10-19</x:v>
+      </x:c>
+      <x:c r="I79" s="66" t="str">
+        <x:v>b929281</x:v>
+      </x:c>
+      <x:c r="J79" s="66" t="str">
+        <x:v>b929281</x:v>
+      </x:c>
+      <x:c r="K79" s="66" t="str">
+        <x:v>src/modules/identity/teams.ts:69-123; src/server.ts:1020-1043</x:v>
+      </x:c>
+      <x:c r="L79" s="66" t="str">
+        <x:v>inviteAccountMember permits OWNER or TECH_ADMIN as inviter; accepts unrestricted requested role including OWNER; API exposes OWNER to TECH_ADMIN.</x:v>
+      </x:c>
+      <x:c r="M79" s="66" t="str">
+        <x:v>A technical admin can grant highest workspace privileges via email invitation.</x:v>
+      </x:c>
+      <x:c r="N79" s="66" t="str">
+        <x:v>Only existing OWNER may invite/assign OWNER; enforce role-grant ceiling inside service function, not only frontend; require recent step-up for ownership changes.</x:v>
+      </x:c>
+      <x:c r="O79" s="66" t="str">
+        <x:v>As TECH_ADMIN POST invite role OWNER returns 403; invites lower authorized roles still work; OWNER with step-up may invite OWNER.</x:v>
+      </x:c>
+      <x:c r="P79" s="66" t="str">
+        <x:v>FORTLESS_AUDIT_BOUNTY_b929281.md</x:v>
+      </x:c>
+      <x:c r="Q79" s="66" t="str">
+        <x:v>https://github.com/trencito42/fortless/blob/b9292811a22159a28a7159deee2c7ff27f41a873/src/modules/identity/teams.ts</x:v>
+      </x:c>
+      <x:c r="R79" s="66" t="str">
+        <x:v>Coding AI</x:v>
+      </x:c>
+      <x:c r="S79" s="66" t="str">
+        <x:v>New code finding; verified statically, no authorized runtime exploit or E2E validation.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="80" ht="50" customHeight="1">
+      <x:c r="A80" s="66" t="str">
+        <x:v>NEW-332</x:v>
+      </x:c>
+      <x:c r="B80" s="66" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C80" s="66" t="str">
+        <x:v>HIGH</x:v>
+      </x:c>
+      <x:c r="D80" s="66" t="str">
+        <x:v>Provisioning</x:v>
+      </x:c>
+      <x:c r="E80" s="66" t="str">
+        <x:v>Live cPanel/VPS routes fall back to in-memory mock adapters</x:v>
+      </x:c>
+      <x:c r="F80" s="66" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="G80" s="66" t="str">
+        <x:v>2026-10-19</x:v>
+      </x:c>
+      <x:c r="H80" s="66" t="str">
+        <x:v>2026-10-19</x:v>
+      </x:c>
+      <x:c r="I80" s="66" t="str">
+        <x:v>b929281</x:v>
+      </x:c>
+      <x:c r="J80" s="66" t="str">
+        <x:v>b929281</x:v>
+      </x:c>
+      <x:c r="K80" s="66" t="str">
+        <x:v>src/modules/outbox/worker.ts:19-34; src/index.ts:44-93</x:v>
+      </x:c>
+      <x:c r="L80" s="66" t="str">
+        <x:v>getAdapterForService returns new MockCpanelAdapter/MockProxmoxAdapter for CPANEL/VPS. bootstrap configures only PterodactylHttpAdapter.</x:v>
+      </x:c>
+      <x:c r="M80" s="66" t="str">
+        <x:v>Order might be fulfilled with a fake remote resource; state shown in Fortless would not exist at provider.</x:v>
+      </x:c>
+      <x:c r="N80" s="66" t="str">
+        <x:v>Inject a provider registry with real configured CpanelHttpAdapter and ProxmoxHttpAdapter; fail closed when unavailable; isolate mocks strictly to test mode.</x:v>
+      </x:c>
+      <x:c r="O80" s="66" t="str">
+        <x:v>In production mode, no CPANEL/VPS event may instantiate Mock*Adapter; integration test checks real provider account/VM and reconciliation.</x:v>
+      </x:c>
+      <x:c r="P80" s="66" t="str">
+        <x:v>FORTLESS_AUDIT_BOUNTY_b929281.md</x:v>
+      </x:c>
+      <x:c r="Q80" s="66" t="str">
+        <x:v>https://github.com/trencito42/fortless/blob/b9292811a22159a28a7159deee2c7ff27f41a873/src/modules/outbox/worker.ts</x:v>
+      </x:c>
+      <x:c r="R80" s="66" t="str">
+        <x:v>Coding AI</x:v>
+      </x:c>
+      <x:c r="S80" s="66" t="str">
+        <x:v>New code finding; verified statically, no authorized runtime exploit or E2E validation.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="81" ht="50" customHeight="1">
+      <x:c r="A81" s="66" t="str">
+        <x:v>NEW-333</x:v>
+      </x:c>
+      <x:c r="B81" s="66" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C81" s="66" t="str">
+        <x:v>HIGH</x:v>
+      </x:c>
+      <x:c r="D81" s="66" t="str">
+        <x:v>Billing</x:v>
+      </x:c>
+      <x:c r="E81" s="66" t="str">
+        <x:v>Fortless cancellation does not cancel Stripe subscription</x:v>
+      </x:c>
+      <x:c r="F81" s="66" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="G81" s="66" t="str">
+        <x:v>2026-10-19</x:v>
+      </x:c>
+      <x:c r="H81" s="66" t="str">
+        <x:v>2026-10-19</x:v>
+      </x:c>
+      <x:c r="I81" s="66" t="str">
+        <x:v>b929281</x:v>
+      </x:c>
+      <x:c r="J81" s="66" t="str">
+        <x:v>b929281</x:v>
+      </x:c>
+      <x:c r="K81" s="66" t="str">
+        <x:v>src/modules/billing/subscriptions.ts:56-132; src/server.ts:1810-1834</x:v>
+      </x:c>
+      <x:c r="L81" s="66" t="str">
+        <x:v>cancelSubscription sets CANCELED or CANCEL_SCHEDULED and auto_renew=0 in SQLite without calling Stripe cancellation/update.</x:v>
+      </x:c>
+      <x:c r="M81" s="66" t="str">
+        <x:v>Customer may see canceled hosting while Stripe keeps charging future invoices.</x:v>
+      </x:c>
+      <x:c r="N81" s="66" t="str">
+        <x:v>Use Stripe API idempotent cancellation at period end or immediate; record PSP state and reconcile asynchronously before final local state.</x:v>
+      </x:c>
+      <x:c r="O81" s="66" t="str">
+        <x:v>Cancel subscription at-period-end and immediate in Stripe test mode; verify Stripe state and Fortless state converge; handle PSP errors/retries.</x:v>
+      </x:c>
+      <x:c r="P81" s="66" t="str">
+        <x:v>FORTLESS_AUDIT_BOUNTY_b929281.md</x:v>
+      </x:c>
+      <x:c r="Q81" s="66" t="str">
+        <x:v>https://github.com/trencito42/fortless/blob/b9292811a22159a28a7159deee2c7ff27f41a873/src/modules/billing/subscriptions.ts</x:v>
+      </x:c>
+      <x:c r="R81" s="66" t="str">
+        <x:v>Coding AI</x:v>
+      </x:c>
+      <x:c r="S81" s="66" t="str">
+        <x:v>New code finding; verified statically, no authorized runtime exploit or E2E validation.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="82" ht="50" customHeight="1">
+      <x:c r="A82" s="66" t="str">
+        <x:v>NEW-334</x:v>
+      </x:c>
+      <x:c r="B82" s="66" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C82" s="66" t="str">
+        <x:v>HIGH</x:v>
+      </x:c>
+      <x:c r="D82" s="66" t="str">
+        <x:v>Billing</x:v>
+      </x:c>
+      <x:c r="E82" s="66" t="str">
+        <x:v>Staff refund modifies local ledger but no PSP refund is made</x:v>
+      </x:c>
+      <x:c r="F82" s="66" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="G82" s="66" t="str">
+        <x:v>2026-10-19</x:v>
+      </x:c>
+      <x:c r="H82" s="66" t="str">
+        <x:v>2026-10-19</x:v>
+      </x:c>
+      <x:c r="I82" s="66" t="str">
+        <x:v>b929281</x:v>
+      </x:c>
+      <x:c r="J82" s="66" t="str">
+        <x:v>b929281</x:v>
+      </x:c>
+      <x:c r="K82" s="66" t="str">
+        <x:v>src/modules/payments/webhooks.ts:521-577; src/server.ts:1920-1950</x:v>
+      </x:c>
+      <x:c r="L82" s="66" t="str">
+        <x:v>processStaffRefund changes invoices and orders locally, calls no Stripe refund API and enqueues no provider teardown for full refunds.</x:v>
+      </x:c>
+      <x:c r="M82" s="66" t="str">
+        <x:v>Customer may be told funds were refunded without receiving money; servers may also remain running.</x:v>
+      </x:c>
+      <x:c r="N82" s="66" t="str">
+        <x:v>Create actual idempotent Stripe refund with PSP refund ID; settle credit note only after accepted/completed provider result and use lifecycle outbox for full refund.</x:v>
+      </x:c>
+      <x:c r="O82" s="66" t="str">
+        <x:v>Staff performs refund of €5: validate Stripe refund exists and amount, exact invoice ledger state, no double refund and service lifecycle matching policy.</x:v>
+      </x:c>
+      <x:c r="P82" s="66" t="str">
+        <x:v>FORTLESS_AUDIT_BOUNTY_b929281.md</x:v>
+      </x:c>
+      <x:c r="Q82" s="66" t="str">
+        <x:v>https://github.com/trencito42/fortless/blob/b9292811a22159a28a7159deee2c7ff27f41a873/src/modules/payments/webhooks.ts</x:v>
+      </x:c>
+      <x:c r="R82" s="66" t="str">
+        <x:v>Coding AI</x:v>
+      </x:c>
+      <x:c r="S82" s="66" t="str">
+        <x:v>New code finding; verified statically, no authorized runtime exploit or E2E validation.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="83" ht="50" customHeight="1">
+      <x:c r="A83" s="66" t="str">
+        <x:v>NEW-335</x:v>
+      </x:c>
+      <x:c r="B83" s="66" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="C83" s="66" t="str">
+        <x:v>HIGH</x:v>
+      </x:c>
+      <x:c r="D83" s="66" t="str">
+        <x:v>Billing</x:v>
+      </x:c>
+      <x:c r="E83" s="66" t="str">
+        <x:v>Multiple partial refunds subtract Stripe cumulative refunded amount repeatedly</x:v>
+      </x:c>
+      <x:c r="F83" s="66" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="G83" s="66" t="str">
+        <x:v>2026-10-19</x:v>
+      </x:c>
+      <x:c r="H83" s="66" t="str">
+        <x:v>2026-10-19</x:v>
+      </x:c>
+      <x:c r="I83" s="66" t="str">
+        <x:v>b929281</x:v>
+      </x:c>
+      <x:c r="J83" s="66" t="str">
+        <x:v>b929281</x:v>
+      </x:c>
+      <x:c r="K83" s="66" t="str">
+        <x:v>src/modules/payments/webhooks.ts:105-145</x:v>
+      </x:c>
+      <x:c r="L83" s="66" t="str">
+        <x:v>charge.refunded uses rawObj.amount_refunded (cumulative on charge) and subtracts it every distinct webhook event; no per-refund delta ledger.</x:v>
+      </x:c>
+      <x:c r="M83" s="66" t="str">
+        <x:v>Two separate partial refunds can overstate total refunded and understate amount paid.</x:v>
+      </x:c>
+      <x:c r="N83" s="66" t="str">
+        <x:v>Reconcile refundable amount via unique refund IDs and delta, or store previous cumulative refunded amount and apply positive difference only.</x:v>
+      </x:c>
+      <x:c r="O83" s="66" t="str">
+        <x:v>Sequential €2 then €3 refunds on €10 charge result in €5 total credited, not €7; replay/out-of-order events have no extra effect.</x:v>
+      </x:c>
+      <x:c r="P83" s="66" t="str">
+        <x:v>FORTLESS_AUDIT_BOUNTY_b929281.md</x:v>
+      </x:c>
+      <x:c r="Q83" s="66" t="str">
+        <x:v>https://github.com/trencito42/fortless/blob/b9292811a22159a28a7159deee2c7ff27f41a873/src/modules/payments/webhooks.ts</x:v>
+      </x:c>
+      <x:c r="R83" s="66" t="str">
+        <x:v>Coding AI</x:v>
+      </x:c>
+      <x:c r="S83" s="66" t="str">
+        <x:v>New code finding; verified statically, no authorized runtime exploit or E2E validation.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="84" ht="50" customHeight="1">
+      <x:c r="A84" s="66" t="str">
+        <x:v>NEW-336</x:v>
+      </x:c>
+      <x:c r="B84" s="66" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="C84" s="66" t="str">
+        <x:v>HIGH</x:v>
+      </x:c>
+      <x:c r="D84" s="66" t="str">
+        <x:v>Billing</x:v>
+      </x:c>
+      <x:c r="E84" s="66" t="str">
+        <x:v>Successful Stripe renewal does not unsuspend an overdue hosting service</x:v>
+      </x:c>
+      <x:c r="F84" s="66" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="G84" s="66" t="str">
+        <x:v>2026-10-19</x:v>
+      </x:c>
+      <x:c r="H84" s="66" t="str">
+        <x:v>2026-10-19</x:v>
+      </x:c>
+      <x:c r="I84" s="66" t="str">
+        <x:v>b929281</x:v>
+      </x:c>
+      <x:c r="J84" s="66" t="str">
+        <x:v>b929281</x:v>
+      </x:c>
+      <x:c r="K84" s="66" t="str">
+        <x:v>src/modules/payments/webhooks.ts:218-246; src/modules/billing/renewal-dunning.ts:235-273</x:v>
+      </x:c>
+      <x:c r="L84" s="66" t="str">
+        <x:v>invoice.paid flips subscription ACTIVE but does not invoke unsuspendService or enqueue reactivation after dunning suspension.</x:v>
+      </x:c>
+      <x:c r="M84" s="66" t="str">
+        <x:v>Customer remains unable to access paid service even after successful retry.</x:v>
+      </x:c>
+      <x:c r="N84" s="66" t="str">
+        <x:v>On matched successful renewal enqueue idempotent unsuspend/reconcile job only when service had been suspended for billing; verify provider state.</x:v>
+      </x:c>
+      <x:c r="O84" s="66" t="str">
+        <x:v>Simulate failed renewal -&gt; grace expiry -&gt; provider suspension -&gt; successful retry; service and provider become active exactly once.</x:v>
+      </x:c>
+      <x:c r="P84" s="66" t="str">
+        <x:v>FORTLESS_AUDIT_BOUNTY_b929281.md</x:v>
+      </x:c>
+      <x:c r="Q84" s="66" t="str">
+        <x:v>https://github.com/trencito42/fortless/blob/b9292811a22159a28a7159deee2c7ff27f41a873/src/modules/payments/webhooks.ts</x:v>
+      </x:c>
+      <x:c r="R84" s="66" t="str">
+        <x:v>Coding AI</x:v>
+      </x:c>
+      <x:c r="S84" s="66" t="str">
+        <x:v>New code finding; verified statically, no authorized runtime exploit or E2E validation.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="85" ht="50" customHeight="1">
+      <x:c r="A85" s="66" t="str">
+        <x:v>NEW-337</x:v>
+      </x:c>
+      <x:c r="B85" s="66" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="C85" s="66" t="str">
+        <x:v>MEDIUM</x:v>
+      </x:c>
+      <x:c r="D85" s="66" t="str">
+        <x:v>Provisioning</x:v>
+      </x:c>
+      <x:c r="E85" s="66" t="str">
+        <x:v>Dead-letter for termination incorrectly reclassifies service as SUSPENDED</x:v>
+      </x:c>
+      <x:c r="F85" s="66" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="G85" s="66" t="str">
+        <x:v>2026-10-19</x:v>
+      </x:c>
+      <x:c r="H85" s="66" t="str">
+        <x:v>2026-10-19</x:v>
+      </x:c>
+      <x:c r="I85" s="66" t="str">
+        <x:v>b929281</x:v>
+      </x:c>
+      <x:c r="J85" s="66" t="str">
+        <x:v>b929281</x:v>
+      </x:c>
+      <x:c r="K85" s="66" t="str">
+        <x:v>src/modules/outbox/worker.ts:145-183</x:v>
+      </x:c>
+      <x:c r="L85" s="66" t="str">
+        <x:v>Worker dead-letter handler unconditionally UPDATE services SET contract_status='SUSPENDED' and logs service.provision_failed for any event type, including service.terminate.v1.</x:v>
+      </x:c>
+      <x:c r="M85" s="66" t="str">
+        <x:v>Failed deletion can restore a terminated service to suspended, obscuring lifecycle and retry obligations.</x:v>
+      </x:c>
+      <x:c r="N85" s="66" t="str">
+        <x:v>Use event-type-specific failure states/audit; deletion failure must stay PENDING_TERMINATION/manual-review, never change to unrelated contract state.</x:v>
+      </x:c>
+      <x:c r="O85" s="66" t="str">
+        <x:v>Force termination provider failure 5 times: service not resurrected as SUSPENDED; actionable failed-delete state/alert remains.</x:v>
+      </x:c>
+      <x:c r="P85" s="66" t="str">
+        <x:v>FORTLESS_AUDIT_BOUNTY_b929281.md</x:v>
+      </x:c>
+      <x:c r="Q85" s="66" t="str">
+        <x:v>https://github.com/trencito42/fortless/blob/b9292811a22159a28a7159deee2c7ff27f41a873/src/modules/outbox/worker.ts</x:v>
+      </x:c>
+      <x:c r="R85" s="66" t="str">
+        <x:v>Coding AI</x:v>
+      </x:c>
+      <x:c r="S85" s="66" t="str">
+        <x:v>New code finding; verified statically, no authorized runtime exploit or E2E validation.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="86" ht="50" customHeight="1">
+      <x:c r="A86" s="66" t="str">
+        <x:v>NEW-338</x:v>
+      </x:c>
+      <x:c r="B86" s="66" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="C86" s="66" t="str">
+        <x:v>HIGH</x:v>
+      </x:c>
+      <x:c r="D86" s="66" t="str">
+        <x:v>Billing</x:v>
+      </x:c>
+      <x:c r="E86" s="66" t="str">
+        <x:v>Order-level Stripe subscription is duplicated across per-service records and amount</x:v>
+      </x:c>
+      <x:c r="F86" s="66" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="G86" s="66" t="str">
+        <x:v>2026-10-19</x:v>
+      </x:c>
+      <x:c r="H86" s="66" t="str">
+        <x:v>2026-10-19</x:v>
+      </x:c>
+      <x:c r="I86" s="66" t="str">
+        <x:v>b929281</x:v>
+      </x:c>
+      <x:c r="J86" s="66" t="str">
+        <x:v>b929281</x:v>
+      </x:c>
+      <x:c r="K86" s="66" t="str">
+        <x:v>src/modules/payments/webhooks.ts:375-462; src/modules/checkout/checkout.ts:198-229</x:v>
+      </x:c>
+      <x:c r="L86" s="66" t="str">
+        <x:v>Checkout creates one Stripe subscription for entire order; webhook inserts one local subscriptions record per service using identical Stripe subscription ID and full order amount as each service renewal_price.</x:v>
+      </x:c>
+      <x:c r="M86" s="66" t="str">
+        <x:v>Renewal totals, cancellations and support actions become ambiguous for multi-service order and may show exaggerated per-service prices.</x:v>
+      </x:c>
+      <x:c r="N86" s="66" t="str">
+        <x:v>Model one PSP subscription per order/invoice with service links and allocations OR one Stripe subscription item per service; persist correct interval and line-item price.</x:v>
+      </x:c>
+      <x:c r="O86" s="66" t="str">
+        <x:v>Buy 2 services in one checkout; one Stripe sub billed correct amount, individual service renewal prices sum to order, cancellation semantics unambiguous.</x:v>
+      </x:c>
+      <x:c r="P86" s="66" t="str">
+        <x:v>FORTLESS_AUDIT_BOUNTY_b929281.md</x:v>
+      </x:c>
+      <x:c r="Q86" s="66" t="str">
+        <x:v>https://github.com/trencito42/fortless/blob/b9292811a22159a28a7159deee2c7ff27f41a873/src/modules/payments/webhooks.ts</x:v>
+      </x:c>
+      <x:c r="R86" s="66" t="str">
+        <x:v>Coding AI</x:v>
+      </x:c>
+      <x:c r="S86" s="66" t="str">
+        <x:v>New code finding; verified statically, no authorized runtime exploit or E2E validation.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5000,7 +5593,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra06e05c174ae46bb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0abc569929324744"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5033,7 +5626,7 @@
     </x:row>
     <x:row r="2" ht="29" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>Engineering control center · baseline 9dacfcb → 6203687 · additional review (same SHA) · 19 October 2026</x:v>
+        <x:v>Engineering control center · baseline 9dacfcb → b929281 · post-fix source review · 19 October 2026</x:v>
       </x:c>
       <x:c r="B2" s="7"/>
       <x:c r="C2" s="7"/>
@@ -5063,22 +5656,22 @@
     </x:row>
     <x:row r="5" ht="31" customHeight="1">
       <x:c r="A5" s="33" t="n">
-        <x:f>COUNTA(Findings!A4:A77)</x:f>
-        <x:v>74</x:v>
+        <x:f>COUNTA(Findings!A4:A86)</x:f>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="B5" s="33"/>
       <x:c r="C5" s="33" t="n">
-        <x:f>COUNTIF(Findings!F4:F77,"OPEN")+COUNTIF(Findings!F4:F77,"REGRESSION")</x:f>
-        <x:v>51</x:v>
+        <x:f>COUNTIF(Findings!F4:F86,"OPEN")+COUNTIF(Findings!F4:F86,"REGRESSION")</x:f>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="D5" s="33"/>
       <x:c r="E5" s="33" t="n">
-        <x:f>COUNTIF(Findings!F4:F77,"FIXED_IN_CODE")</x:f>
-        <x:v>7</x:v>
+        <x:f>COUNTIF(Findings!F4:F86,"FIXED_IN_CODE")</x:f>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="F5" s="33"/>
       <x:c r="G5" s="33" t="n">
-        <x:f>COUNTIF(Findings!F4:F77,"CLOSED")+COUNTIF(Findings!F4:F77,"TESTED")</x:f>
+        <x:f>COUNTIF(Findings!F4:F86,"CLOSED")+COUNTIF(Findings!F4:F86,"TESTED")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="H5" s="33"/>
@@ -5111,8 +5704,8 @@
         <x:v>OPEN</x:v>
       </x:c>
       <x:c r="B10" t="n">
-        <x:f>COUNTIF(Findings!F4:F77,A10)</x:f>
-        <x:v>51</x:v>
+        <x:f>COUNTIF(Findings!F4:F86,A10)</x:f>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="C10" t="str">
         <x:v>Priority</x:v>
@@ -5121,9 +5714,9 @@
         <x:v>Count</x:v>
       </x:c>
       <x:c r="F10" s="43" t="str">
-        <x:v>NOT CLEARED FOR PUBLIC PAID LAUNCH
-Static code findings remain, provider E2E and Stripe billing lifecycles not independently tested.
-Do not close a ticket based only on an AI statement or commit title.</x:v>
+        <x:v>NOT CLEARED FOR REAL PAYMENTS
+High-impact billing and provider consistency defects remain.
+Static review only. Require real PSP/provider E2E and verified backups before launch.</x:v>
       </x:c>
       <x:c r="G10" s="43"/>
       <x:c r="H10" s="43"/>
@@ -5133,15 +5726,15 @@
         <x:v>PARTIAL</x:v>
       </x:c>
       <x:c r="B11" t="n">
-        <x:f>COUNTIF(Findings!F4:F77,A11)</x:f>
-        <x:v>3</x:v>
+        <x:f>COUNTIF(Findings!F4:F86,A11)</x:f>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="C11" t="str">
         <x:v>P0</x:v>
       </x:c>
       <x:c r="D11" t="n">
-        <x:f>COUNTIF(Findings!B4:B77,C11)</x:f>
-        <x:v>26</x:v>
+        <x:f>COUNTIF(Findings!B4:B86,C11)</x:f>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="F11" s="43"/>
       <x:c r="G11" s="43"/>
@@ -5152,15 +5745,15 @@
         <x:v>NEEDS_VERIFICATION</x:v>
       </x:c>
       <x:c r="B12" t="n">
-        <x:f>COUNTIF(Findings!F4:F77,A12)</x:f>
+        <x:f>COUNTIF(Findings!F4:F86,A12)</x:f>
         <x:v>11</x:v>
       </x:c>
       <x:c r="C12" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="D12" t="n">
-        <x:f>COUNTIF(Findings!B4:B77,C12)</x:f>
-        <x:v>46</x:v>
+        <x:f>COUNTIF(Findings!B4:B86,C12)</x:f>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="F12" s="43"/>
       <x:c r="G12" s="43"/>
@@ -5171,14 +5764,14 @@
         <x:v>POLICY_DECISION</x:v>
       </x:c>
       <x:c r="B13" t="n">
-        <x:f>COUNTIF(Findings!F4:F77,A13)</x:f>
+        <x:f>COUNTIF(Findings!F4:F86,A13)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="C13" t="str">
         <x:v>P2</x:v>
       </x:c>
       <x:c r="D13" t="n">
-        <x:f>COUNTIF(Findings!B4:B77,C13)</x:f>
+        <x:f>COUNTIF(Findings!B4:B86,C13)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="F13" s="43"/>
@@ -5190,8 +5783,8 @@
         <x:v>FIXED_IN_CODE</x:v>
       </x:c>
       <x:c r="B14" t="n">
-        <x:f>COUNTIF(Findings!F4:F77,A14)</x:f>
-        <x:v>7</x:v>
+        <x:f>COUNTIF(Findings!F4:F86,A14)</x:f>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="F14" s="43"/>
       <x:c r="G14" s="43"/>
@@ -5202,7 +5795,7 @@
         <x:v>TESTED</x:v>
       </x:c>
       <x:c r="B15" t="n">
-        <x:f>COUNTIF(Findings!F4:F77,A15)</x:f>
+        <x:f>COUNTIF(Findings!F4:F86,A15)</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -5211,7 +5804,7 @@
         <x:v>CLOSED</x:v>
       </x:c>
       <x:c r="B16" t="n">
-        <x:f>COUNTIF(Findings!F4:F77,A16)</x:f>
+        <x:f>COUNTIF(Findings!F4:F86,A16)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F16" t="str">
@@ -5223,11 +5816,11 @@
         <x:v>REGRESSION</x:v>
       </x:c>
       <x:c r="B17" t="n">
-        <x:f>COUNTIF(Findings!F4:F77,A17)</x:f>
+        <x:f>COUNTIF(Findings!F4:F86,A17)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F17" s="51" t="str">
-        <x:v>620368742f1d</x:v>
+        <x:v>b9292811a221</x:v>
       </x:c>
       <x:c r="G17" s="51"/>
       <x:c r="H17" s="51"/>
@@ -5968,7 +6561,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R713fc674367a4f18"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R690f713a26384c84"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6163,6 +6756,26 @@
       </x:c>
       <x:c r="F10" s="18" t="str">
         <x:v>Same HEAD 6203687; not a new push</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" t="str">
+        <x:v>2026-10-19 04:02</x:v>
+      </x:c>
+      <x:c r="B11" t="str">
+        <x:v>b929281</x:v>
+      </x:c>
+      <x:c r="C11" t="str">
+        <x:v>Agent's audit delta security/billing/UI corrections</x:v>
+      </x:c>
+      <x:c r="D11" t="str">
+        <x:v>Independent static recheck: 21 status transitions; 9 new findings NEW-330…338</x:v>
+      </x:c>
+      <x:c r="E11" t="str">
+        <x:v>STATIC_SOURCE_ONLY</x:v>
+      </x:c>
+      <x:c r="F11" t="str">
+        <x:v>b9292811a22159a28a7159deee2c7ff27f41a873</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -6462,6 +7075,489 @@
         <x:v>Terminated service no longer displays Manage</x:v>
       </x:c>
     </x:row>
+    <x:row r="14" ht="27" customHeight="1">
+      <x:c r="A14" t="str">
+        <x:v>2026-10-19</x:v>
+      </x:c>
+      <x:c r="B14" t="str">
+        <x:v>b929281</x:v>
+      </x:c>
+      <x:c r="C14" t="str">
+        <x:v>SEC-04</x:v>
+      </x:c>
+      <x:c r="D14" t="str">
+        <x:v>PARTIAL</x:v>
+      </x:c>
+      <x:c r="E14" t="str">
+        <x:v>FIXED_IN_CODE</x:v>
+      </x:c>
+      <x:c r="F14" t="str">
+        <x:v>Static source inspection</x:v>
+      </x:c>
+      <x:c r="G14" t="str">
+        <x:v>Pending-MFA 15-min TTL and account-wide failures in auth.ts; requires runtime test.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="27" customHeight="1">
+      <x:c r="A15" t="str">
+        <x:v>2026-10-19</x:v>
+      </x:c>
+      <x:c r="B15" t="str">
+        <x:v>b929281</x:v>
+      </x:c>
+      <x:c r="C15" t="str">
+        <x:v>FTL-SEC-201</x:v>
+      </x:c>
+      <x:c r="D15" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="E15" t="str">
+        <x:v>FIXED_IN_CODE</x:v>
+      </x:c>
+      <x:c r="F15" t="str">
+        <x:v>Static source inspection</x:v>
+      </x:c>
+      <x:c r="G15" t="str">
+        <x:v>Confirmed factor remains active; pending_secret_encrypted used for replacement.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="27" customHeight="1">
+      <x:c r="A16" t="str">
+        <x:v>2026-10-19</x:v>
+      </x:c>
+      <x:c r="B16" t="str">
+        <x:v>b929281</x:v>
+      </x:c>
+      <x:c r="C16" t="str">
+        <x:v>FTL-SEC-202</x:v>
+      </x:c>
+      <x:c r="D16" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="E16" t="str">
+        <x:v>FIXED_IN_CODE</x:v>
+      </x:c>
+      <x:c r="F16" t="str">
+        <x:v>Static source inspection</x:v>
+      </x:c>
+      <x:c r="G16" t="str">
+        <x:v>MFA failures now queried by user_id across all pending sessions.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="27" customHeight="1">
+      <x:c r="A17" t="str">
+        <x:v>2026-10-19</x:v>
+      </x:c>
+      <x:c r="B17" t="str">
+        <x:v>b929281</x:v>
+      </x:c>
+      <x:c r="C17" t="str">
+        <x:v>FTL-SEC-203</x:v>
+      </x:c>
+      <x:c r="D17" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="E17" t="str">
+        <x:v>FIXED_IN_CODE</x:v>
+      </x:c>
+      <x:c r="F17" t="str">
+        <x:v>Static source inspection</x:v>
+      </x:c>
+      <x:c r="G17" t="str">
+        <x:v>Recovery-code regeneration protected by requireRecentStepUp.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="27" customHeight="1">
+      <x:c r="A18" t="str">
+        <x:v>2026-10-19</x:v>
+      </x:c>
+      <x:c r="B18" t="str">
+        <x:v>b929281</x:v>
+      </x:c>
+      <x:c r="C18" t="str">
+        <x:v>FTL-SEC-204</x:v>
+      </x:c>
+      <x:c r="D18" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="E18" t="str">
+        <x:v>FIXED_IN_CODE</x:v>
+      </x:c>
+      <x:c r="F18" t="str">
+        <x:v>Static source inspection</x:v>
+      </x:c>
+      <x:c r="G18" t="str">
+        <x:v>Recovery codes now 128-bit generated from randomBytes(16).</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="27" customHeight="1">
+      <x:c r="A19" t="str">
+        <x:v>2026-10-19</x:v>
+      </x:c>
+      <x:c r="B19" t="str">
+        <x:v>b929281</x:v>
+      </x:c>
+      <x:c r="C19" t="str">
+        <x:v>FTL-SEC-205</x:v>
+      </x:c>
+      <x:c r="D19" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="E19" t="str">
+        <x:v>FIXED_IN_CODE</x:v>
+      </x:c>
+      <x:c r="F19" t="str">
+        <x:v>Static source inspection</x:v>
+      </x:c>
+      <x:c r="G19" t="str">
+        <x:v>isLoginThrottled now counts 10 failures account-wide independent of IP.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="27" customHeight="1">
+      <x:c r="A20" t="str">
+        <x:v>2026-10-19</x:v>
+      </x:c>
+      <x:c r="B20" t="str">
+        <x:v>b929281</x:v>
+      </x:c>
+      <x:c r="C20" t="str">
+        <x:v>FTL-BILL-201</x:v>
+      </x:c>
+      <x:c r="D20" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="E20" t="str">
+        <x:v>PARTIAL</x:v>
+      </x:c>
+      <x:c r="F20" t="str">
+        <x:v>Static source inspection</x:v>
+      </x:c>
+      <x:c r="G20" t="str">
+        <x:v>Stripe recurring interval mapped correctly; webhook still persists local subscriptions as MONTHLY.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="27" customHeight="1">
+      <x:c r="A21" t="str">
+        <x:v>2026-10-19</x:v>
+      </x:c>
+      <x:c r="B21" t="str">
+        <x:v>b929281</x:v>
+      </x:c>
+      <x:c r="C21" t="str">
+        <x:v>FTL-BILL-202</x:v>
+      </x:c>
+      <x:c r="D21" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="E21" t="str">
+        <x:v>PARTIAL</x:v>
+      </x:c>
+      <x:c r="F21" t="str">
+        <x:v>Static source inspection</x:v>
+      </x:c>
+      <x:c r="G21" t="str">
+        <x:v>Refund/dispute webhook enqueues suspend/terminate actions; staff refund path still bypasses PSP/provider.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="27" customHeight="1">
+      <x:c r="A22" t="str">
+        <x:v>2026-10-19</x:v>
+      </x:c>
+      <x:c r="B22" t="str">
+        <x:v>b929281</x:v>
+      </x:c>
+      <x:c r="C22" t="str">
+        <x:v>FTL-BILL-203</x:v>
+      </x:c>
+      <x:c r="D22" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="E22" t="str">
+        <x:v>FIXED_IN_CODE</x:v>
+      </x:c>
+      <x:c r="F22" t="str">
+        <x:v>Static source inspection</x:v>
+      </x:c>
+      <x:c r="G22" t="str">
+        <x:v>Webhook checks payment_attempts.status/order.status before repeated fulfillment.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="27" customHeight="1">
+      <x:c r="A23" t="str">
+        <x:v>2026-10-19</x:v>
+      </x:c>
+      <x:c r="B23" t="str">
+        <x:v>b929281</x:v>
+      </x:c>
+      <x:c r="C23" t="str">
+        <x:v>FTL-BILL-204</x:v>
+      </x:c>
+      <x:c r="D23" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="E23" t="str">
+        <x:v>PARTIAL</x:v>
+      </x:c>
+      <x:c r="F23" t="str">
+        <x:v>Static source inspection</x:v>
+      </x:c>
+      <x:c r="G23" t="str">
+        <x:v>Real payment_intent IDs stored; invoice.paid settlement scopes invoices by account, not Stripe invoice.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="27" customHeight="1">
+      <x:c r="A24" t="str">
+        <x:v>2026-10-19</x:v>
+      </x:c>
+      <x:c r="B24" t="str">
+        <x:v>b929281</x:v>
+      </x:c>
+      <x:c r="C24" t="str">
+        <x:v>FTL-BILL-205</x:v>
+      </x:c>
+      <x:c r="D24" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="E24" t="str">
+        <x:v>PARTIAL</x:v>
+      </x:c>
+      <x:c r="F24" t="str">
+        <x:v>Static source inspection</x:v>
+      </x:c>
+      <x:c r="G24" t="str">
+        <x:v>Stripe subscriptions exempted from local dunning; invoice.paid wrongly settles all account invoices.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="27" customHeight="1">
+      <x:c r="A25" t="str">
+        <x:v>2026-10-19</x:v>
+      </x:c>
+      <x:c r="B25" t="str">
+        <x:v>b929281</x:v>
+      </x:c>
+      <x:c r="C25" t="str">
+        <x:v>FTL-PROV-201</x:v>
+      </x:c>
+      <x:c r="D25" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="E25" t="str">
+        <x:v>PARTIAL</x:v>
+      </x:c>
+      <x:c r="F25" t="str">
+        <x:v>Static source inspection</x:v>
+      </x:c>
+      <x:c r="G25" t="str">
+        <x:v>Dispatch by provider_type added, but CPANEL/VPS dispatch still constructs mock adapters in worker.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="27" customHeight="1">
+      <x:c r="A26" t="str">
+        <x:v>2026-10-19</x:v>
+      </x:c>
+      <x:c r="B26" t="str">
+        <x:v>b929281</x:v>
+      </x:c>
+      <x:c r="C26" t="str">
+        <x:v>FTL-PROV-202</x:v>
+      </x:c>
+      <x:c r="D26" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="E26" t="str">
+        <x:v>PARTIAL</x:v>
+      </x:c>
+      <x:c r="F26" t="str">
+        <x:v>Static source inspection</x:v>
+      </x:c>
+      <x:c r="G26" t="str">
+        <x:v>Hardcoded node_fra_01 removed; fallback still chooses wrong region/no-capacity nodes.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="27" customHeight="1">
+      <x:c r="A27" t="str">
+        <x:v>2026-10-19</x:v>
+      </x:c>
+      <x:c r="B27" t="str">
+        <x:v>b929281</x:v>
+      </x:c>
+      <x:c r="C27" t="str">
+        <x:v>FTL-PROV-203</x:v>
+      </x:c>
+      <x:c r="D27" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="E27" t="str">
+        <x:v>FIXED_IN_CODE</x:v>
+      </x:c>
+      <x:c r="F27" t="str">
+        <x:v>Static source inspection</x:v>
+      </x:c>
+      <x:c r="G27" t="str">
+        <x:v>Worker now atomically reserves capacity with conditional UPDATE.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="27" customHeight="1">
+      <x:c r="A28" t="str">
+        <x:v>2026-10-19</x:v>
+      </x:c>
+      <x:c r="B28" t="str">
+        <x:v>b929281</x:v>
+      </x:c>
+      <x:c r="C28" t="str">
+        <x:v>FTL-DNS-201</x:v>
+      </x:c>
+      <x:c r="D28" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="E28" t="str">
+        <x:v>PARTIAL</x:v>
+      </x:c>
+      <x:c r="F28" t="str">
+        <x:v>Static source inspection</x:v>
+      </x:c>
+      <x:c r="G28" t="str">
+        <x:v>Search discloses LOCAL_ZONE_AVAILABLE, but still returns available:true without registrar check.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="27" customHeight="1">
+      <x:c r="A29" t="str">
+        <x:v>2026-10-19</x:v>
+      </x:c>
+      <x:c r="B29" t="str">
+        <x:v>b929281</x:v>
+      </x:c>
+      <x:c r="C29" t="str">
+        <x:v>FTL-DNS-202</x:v>
+      </x:c>
+      <x:c r="D29" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="E29" t="str">
+        <x:v>PARTIAL</x:v>
+      </x:c>
+      <x:c r="F29" t="str">
+        <x:v>Static source inspection</x:v>
+      </x:c>
+      <x:c r="G29" t="str">
+        <x:v>Zone has pending/delegation distinction; authoritative DNS/registrar integration not verified.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="27" customHeight="1">
+      <x:c r="A30" t="str">
+        <x:v>2026-10-19</x:v>
+      </x:c>
+      <x:c r="B30" t="str">
+        <x:v>b929281</x:v>
+      </x:c>
+      <x:c r="C30" t="str">
+        <x:v>FTL-UI-201</x:v>
+      </x:c>
+      <x:c r="D30" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="E30" t="str">
+        <x:v>FIXED_IN_CODE</x:v>
+      </x:c>
+      <x:c r="F30" t="str">
+        <x:v>Static source inspection</x:v>
+      </x:c>
+      <x:c r="G30" t="str">
+        <x:v>Service list checks user_can_control, detailed page checks explicit permissions; runtime E2E needed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="27" customHeight="1">
+      <x:c r="A31" t="str">
+        <x:v>2026-10-19</x:v>
+      </x:c>
+      <x:c r="B31" t="str">
+        <x:v>b929281</x:v>
+      </x:c>
+      <x:c r="C31" t="str">
+        <x:v>FTL-UI-202</x:v>
+      </x:c>
+      <x:c r="D31" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="E31" t="str">
+        <x:v>FIXED_IN_CODE</x:v>
+      </x:c>
+      <x:c r="F31" t="str">
+        <x:v>Static source inspection</x:v>
+      </x:c>
+      <x:c r="G31" t="str">
+        <x:v>Service details filter provider tabs by capabilities and permissions.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="27" customHeight="1">
+      <x:c r="A32" t="str">
+        <x:v>2026-10-19</x:v>
+      </x:c>
+      <x:c r="B32" t="str">
+        <x:v>b929281</x:v>
+      </x:c>
+      <x:c r="C32" t="str">
+        <x:v>FTL-UI-203</x:v>
+      </x:c>
+      <x:c r="D32" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="E32" t="str">
+        <x:v>PARTIAL</x:v>
+      </x:c>
+      <x:c r="F32" t="str">
+        <x:v>Static source inspection</x:v>
+      </x:c>
+      <x:c r="G32" t="str">
+        <x:v>Router has sequence and AbortController; async page fetches do not consistently use signal guard.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="27" customHeight="1">
+      <x:c r="A33" t="str">
+        <x:v>2026-10-19</x:v>
+      </x:c>
+      <x:c r="B33" t="str">
+        <x:v>b929281</x:v>
+      </x:c>
+      <x:c r="C33" t="str">
+        <x:v>FTL-UI-204</x:v>
+      </x:c>
+      <x:c r="D33" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="E33" t="str">
+        <x:v>PARTIAL</x:v>
+      </x:c>
+      <x:c r="F33" t="str">
+        <x:v>Static source inspection</x:v>
+      </x:c>
+      <x:c r="G33" t="str">
+        <x:v>24 route definitions present in verify-views.py, but no authenticated fixture/pixel reference comparison.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="27" customHeight="1">
+      <x:c r="A34" t="str">
+        <x:v>2026-10-19</x:v>
+      </x:c>
+      <x:c r="B34" t="str">
+        <x:v>b929281</x:v>
+      </x:c>
+      <x:c r="C34" t="str">
+        <x:v>FTL-UI-206</x:v>
+      </x:c>
+      <x:c r="D34" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="E34" t="str">
+        <x:v>PARTIAL</x:v>
+      </x:c>
+      <x:c r="F34" t="str">
+        <x:v>Static source inspection</x:v>
+      </x:c>
+      <x:c r="G34" t="str">
+        <x:v>Buttons account for contract/runtime status but per-button action permission and provider feedback remain incomplete.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:G1"/>
@@ -6917,4 +8013,516 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="28" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="30" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="40" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="47" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="27" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="33" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="32" customHeight="1">
+      <x:c r="A1" s="74" t="str">
+        <x:v>FORTLESS  /  RISK-BASED MFA &amp; STEP-UP MATRIX</x:v>
+      </x:c>
+      <x:c r="B1" s="74"/>
+      <x:c r="C1" s="74"/>
+      <x:c r="D1" s="74"/>
+      <x:c r="E1" s="74"/>
+      <x:c r="F1" s="74"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" t="str">
+        <x:v>Recommend strong verification only for identity, ownership, finance, destructive changes. Keep routine server operations frictionless.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="30" customHeight="1">
+      <x:c r="A4" s="76" t="str">
+        <x:v>Action / endpoint</x:v>
+      </x:c>
+      <x:c r="B4" s="76" t="str">
+        <x:v>Policy</x:v>
+      </x:c>
+      <x:c r="C4" s="76" t="str">
+        <x:v>Existing observed control</x:v>
+      </x:c>
+      <x:c r="D4" s="76" t="str">
+        <x:v>Gap / change needed</x:v>
+      </x:c>
+      <x:c r="E4" s="76" t="str">
+        <x:v>Reason</x:v>
+      </x:c>
+      <x:c r="F4" s="76" t="str">
+        <x:v>Tracking / code</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="39" customHeight="1">
+      <x:c r="A5" s="66" t="str">
+        <x:v>Staff admin access</x:v>
+      </x:c>
+      <x:c r="B5" s="66" t="str">
+        <x:v>MFA mandatory</x:v>
+      </x:c>
+      <x:c r="C5" s="66" t="str">
+        <x:v>Staff guard requires verified MFA</x:v>
+      </x:c>
+      <x:c r="D5" s="66" t="str">
+        <x:v>Test direct API and SSO consistency</x:v>
+      </x:c>
+      <x:c r="E5" s="66" t="str">
+        <x:v>Privileged all-tenant surface</x:v>
+      </x:c>
+      <x:c r="F5" s="66" t="str">
+        <x:v>src/server.ts requireStaff</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="39" customHeight="1">
+      <x:c r="A6" s="66" t="str">
+        <x:v>Staff refund</x:v>
+      </x:c>
+      <x:c r="B6" s="66" t="str">
+        <x:v>Recent step-up mandatory</x:v>
+      </x:c>
+      <x:c r="C6" s="66" t="str">
+        <x:v>requireRecentStepUp in refund route</x:v>
+      </x:c>
+      <x:c r="D6" s="66" t="str">
+        <x:v>Keep, enforce PSP refund idempotence</x:v>
+      </x:c>
+      <x:c r="E6" s="66" t="str">
+        <x:v>Financial mutation</x:v>
+      </x:c>
+      <x:c r="F6" s="66" t="str">
+        <x:v>src/server.ts:1920; NEW-334</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="39" customHeight="1">
+      <x:c r="A7" s="66" t="str">
+        <x:v>Staff service terminate / relink</x:v>
+      </x:c>
+      <x:c r="B7" s="66" t="str">
+        <x:v>Recent step-up mandatory</x:v>
+      </x:c>
+      <x:c r="C7" s="66" t="str">
+        <x:v>Admin routes guarded</x:v>
+      </x:c>
+      <x:c r="D7" s="66" t="str">
+        <x:v>Keep; provider deletion must reconcile</x:v>
+      </x:c>
+      <x:c r="E7" s="66" t="str">
+        <x:v>Permanent destructive change</x:v>
+      </x:c>
+      <x:c r="F7" s="66" t="str">
+        <x:v>src/server.ts; NEW-337</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="39" customHeight="1">
+      <x:c r="A8" s="66" t="str">
+        <x:v>Invite/promote OWNER</x:v>
+      </x:c>
+      <x:c r="B8" s="66" t="str">
+        <x:v>Owner-only + fresh step-up</x:v>
+      </x:c>
+      <x:c r="C8" s="66" t="str">
+        <x:v>TECH_ADMIN may currently invite OWNER</x:v>
+      </x:c>
+      <x:c r="D8" s="66" t="str">
+        <x:v>Deny upward grant; step-up owner changes</x:v>
+      </x:c>
+      <x:c r="E8" s="66" t="str">
+        <x:v>Privilege escalation</x:v>
+      </x:c>
+      <x:c r="F8" s="66" t="str">
+        <x:v>NEW-331</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="39" customHeight="1">
+      <x:c r="A9" s="66" t="str">
+        <x:v>Register / delete passkeys</x:v>
+      </x:c>
+      <x:c r="B9" s="66" t="str">
+        <x:v>Recent step-up</x:v>
+      </x:c>
+      <x:c r="C9" s="66" t="str">
+        <x:v>Authentication only on passkey routes</x:v>
+      </x:c>
+      <x:c r="D9" s="66" t="str">
+        <x:v>Require recent auth or UV; alert user</x:v>
+      </x:c>
+      <x:c r="E9" s="66" t="str">
+        <x:v>Future account takeover</x:v>
+      </x:c>
+      <x:c r="F9" s="66" t="str">
+        <x:v>NEW-306</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="39" customHeight="1">
+      <x:c r="A10" s="66" t="str">
+        <x:v>Reset/replace MFA</x:v>
+      </x:c>
+      <x:c r="B10" s="66" t="str">
+        <x:v>Recent step-up + notify</x:v>
+      </x:c>
+      <x:c r="C10" s="66" t="str">
+        <x:v>TOTP replacement step-up; recovery regenerate step-up</x:v>
+      </x:c>
+      <x:c r="D10" s="66" t="str">
+        <x:v>Test session revocation and step-up replay</x:v>
+      </x:c>
+      <x:c r="E10" s="66" t="str">
+        <x:v>Security factor change</x:v>
+      </x:c>
+      <x:c r="F10" s="66" t="str">
+        <x:v>FTL-SEC-201/203</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="39" customHeight="1">
+      <x:c r="A11" s="66" t="str">
+        <x:v>Disable MFA</x:v>
+      </x:c>
+      <x:c r="B11" s="66" t="str">
+        <x:v>Password + current MFA; alerts</x:v>
+      </x:c>
+      <x:c r="C11" s="66" t="str">
+        <x:v>Password + TOTP checked</x:v>
+      </x:c>
+      <x:c r="D11" s="66" t="str">
+        <x:v>Review session revocation; staff policy</x:v>
+      </x:c>
+      <x:c r="E11" s="66" t="str">
+        <x:v>Weakens account protection</x:v>
+      </x:c>
+      <x:c r="F11" s="66" t="str">
+        <x:v>src/modules/identity/auth.ts</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="39" customHeight="1">
+      <x:c r="A12" s="66" t="str">
+        <x:v>Workspace invite TECH_ADMIN</x:v>
+      </x:c>
+      <x:c r="B12" s="66" t="str">
+        <x:v>Owner or allowed tech admin + step-up</x:v>
+      </x:c>
+      <x:c r="C12" s="66" t="str">
+        <x:v>Only role check</x:v>
+      </x:c>
+      <x:c r="D12" s="66" t="str">
+        <x:v>Add step-up for privileged invitations</x:v>
+      </x:c>
+      <x:c r="E12" s="66" t="str">
+        <x:v>Role management</x:v>
+      </x:c>
+      <x:c r="F12" s="66" t="str">
+        <x:v>src/modules/identity/teams.ts</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="39" customHeight="1">
+      <x:c r="A13" s="66" t="str">
+        <x:v>Change PSP/provider API keys</x:v>
+      </x:c>
+      <x:c r="B13" s="66" t="str">
+        <x:v>Fresh step-up + confirmation</x:v>
+      </x:c>
+      <x:c r="C13" s="66" t="str">
+        <x:v>Config mostly via server env</x:v>
+      </x:c>
+      <x:c r="D13" s="66" t="str">
+        <x:v>Gate any future admin UI and dual confirmation</x:v>
+      </x:c>
+      <x:c r="E13" s="66" t="str">
+        <x:v>Can control all infrastructure / money</x:v>
+      </x:c>
+      <x:c r="F13" s="66" t="str">
+        <x:v>Launch controls</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="39" customHeight="1">
+      <x:c r="A14" s="66" t="str">
+        <x:v>Backup restore / reinstall</x:v>
+      </x:c>
+      <x:c r="B14" s="66" t="str">
+        <x:v>Confirmation; optional recent step-up</x:v>
+      </x:c>
+      <x:c r="C14" s="66" t="str">
+        <x:v>Permission checks on API</x:v>
+      </x:c>
+      <x:c r="D14" s="66" t="str">
+        <x:v>Use step-up on destructive restore, not listing</x:v>
+      </x:c>
+      <x:c r="E14" s="66" t="str">
+        <x:v>Destructive service operation</x:v>
+      </x:c>
+      <x:c r="F14" s="66" t="str">
+        <x:v>src/modules/provisioning/server-panel.ts</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="39" customHeight="1">
+      <x:c r="A15" s="66" t="str">
+        <x:v>Routine start/stop/console</x:v>
+      </x:c>
+      <x:c r="B15" s="66" t="str">
+        <x:v>No additional MFA per click</x:v>
+      </x:c>
+      <x:c r="C15" s="66" t="str">
+        <x:v>Session + per-service permissions</x:v>
+      </x:c>
+      <x:c r="D15" s="66" t="str">
+        <x:v>Keep quick and responsive</x:v>
+      </x:c>
+      <x:c r="E15" s="66" t="str">
+        <x:v>UX without unnecessary friction</x:v>
+      </x:c>
+      <x:c r="F15" s="66" t="str">
+        <x:v>src/modules/provisioning/service-access.ts</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="39" customHeight="1">
+      <x:c r="A16" s="66" t="str">
+        <x:v>Normal checkout</x:v>
+      </x:c>
+      <x:c r="B16" s="66" t="str">
+        <x:v>SCA through Stripe, no duplicate TOTP</x:v>
+      </x:c>
+      <x:c r="C16" s="66" t="str">
+        <x:v>Stripe Checkout handles payment auth</x:v>
+      </x:c>
+      <x:c r="D16" s="66" t="str">
+        <x:v>Avoid double MFA unless suspicious session</x:v>
+      </x:c>
+      <x:c r="E16" s="66" t="str">
+        <x:v>Reduce checkout friction</x:v>
+      </x:c>
+      <x:c r="F16" s="66" t="str">
+        <x:v>src/modules/checkout/checkout.ts</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="39" customHeight="1">
+      <x:c r="A17" s="66" t="str">
+        <x:v>Staff passkey sign-in</x:v>
+      </x:c>
+      <x:c r="B17" s="66" t="str">
+        <x:v>Require authenticator user verification</x:v>
+      </x:c>
+      <x:c r="C17" s="66" t="str">
+        <x:v>Policy userVerification preferred</x:v>
+      </x:c>
+      <x:c r="D17" s="66" t="str">
+        <x:v>Upgrade privileged authentication policy to required</x:v>
+      </x:c>
+      <x:c r="E17" s="66" t="str">
+        <x:v>Phishing-resistant control</x:v>
+      </x:c>
+      <x:c r="F17" s="66" t="str">
+        <x:v>NEW-307</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:F1"/>
+    <x:mergeCell ref="A2:F2"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="10" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="30" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="58" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="49" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="32" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="22" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="32" customHeight="1">
+      <x:c r="A1" s="74" t="str">
+        <x:v>FORTLESS  /  SINGLE-OPERATOR HOSTING RELEASE GATES</x:v>
+      </x:c>
+      <x:c r="B1" s="74"/>
+      <x:c r="C1" s="74"/>
+      <x:c r="D1" s="74"/>
+      <x:c r="E1" s="74"/>
+      <x:c r="F1" s="74"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" t="str">
+        <x:v>Designed for a controlled commercial hosting launch, not hyperscale. Ship Pterodactyl first; disable unverified providers until live integration passes.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="32" customHeight="1">
+      <x:c r="A4" s="76" t="str">
+        <x:v>Phase</x:v>
+      </x:c>
+      <x:c r="B4" s="76" t="str">
+        <x:v>Release gate</x:v>
+      </x:c>
+      <x:c r="C4" s="76" t="str">
+        <x:v>Exit criterion (not just AI green text)</x:v>
+      </x:c>
+      <x:c r="D4" s="76" t="str">
+        <x:v>Evidence required</x:v>
+      </x:c>
+      <x:c r="E4" s="76" t="str">
+        <x:v>Scope</x:v>
+      </x:c>
+      <x:c r="F4" s="76" t="str">
+        <x:v>State</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="64" customHeight="1">
+      <x:c r="A5" s="66" t="str">
+        <x:v>01</x:v>
+      </x:c>
+      <x:c r="B5" s="66" t="str">
+        <x:v>Stop incorrect money flow</x:v>
+      </x:c>
+      <x:c r="C5" s="66" t="str">
+        <x:v>Stripe invoice/payment/subscription/refund/cancel exactly matched; no double settlement or charging after cancel</x:v>
+      </x:c>
+      <x:c r="D5" s="66" t="str">
+        <x:v>Integration tests + Stripe test mode webhook replay + sample invoices</x:v>
+      </x:c>
+      <x:c r="E5" s="66" t="str">
+        <x:v>Billing, credit notes, VAT, pricing</x:v>
+      </x:c>
+      <x:c r="F5" s="66" t="str">
+        <x:v>BLOCKED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="64" customHeight="1">
+      <x:c r="A6" s="66" t="str">
+        <x:v>02</x:v>
+      </x:c>
+      <x:c r="B6" s="66" t="str">
+        <x:v>Fix privilege boundaries</x:v>
+      </x:c>
+      <x:c r="C6" s="66" t="str">
+        <x:v>OWNER roles ungrantable by TECH_ADMIN; all service operations pass two-account RBAC tests</x:v>
+      </x:c>
+      <x:c r="D6" s="66" t="str">
+        <x:v>Test matrix across OWNER/TECH_ADMIN/BILLING/VIEWER/shared presets</x:v>
+      </x:c>
+      <x:c r="E6" s="66" t="str">
+        <x:v>Auth, sessions, service permissions</x:v>
+      </x:c>
+      <x:c r="F6" s="66" t="str">
+        <x:v>BLOCKED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="64" customHeight="1">
+      <x:c r="A7" s="66" t="str">
+        <x:v>03</x:v>
+      </x:c>
+      <x:c r="B7" s="66" t="str">
+        <x:v>Real provider operations only</x:v>
+      </x:c>
+      <x:c r="C7" s="66" t="str">
+        <x:v>No mock provisioning in live; one successful create, suspend, resume, delete, retry &amp; reconcile for each published provider</x:v>
+      </x:c>
+      <x:c r="D7" s="66" t="str">
+        <x:v>Provider sandbox/live test resources + logs</x:v>
+      </x:c>
+      <x:c r="E7" s="66" t="str">
+        <x:v>Pterodactyl core; cPanel/VPS gated</x:v>
+      </x:c>
+      <x:c r="F7" s="66" t="str">
+        <x:v>BLOCKED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="64" customHeight="1">
+      <x:c r="A8" s="66" t="str">
+        <x:v>04</x:v>
+      </x:c>
+      <x:c r="B8" s="66" t="str">
+        <x:v>State machine &amp; reconciliation</x:v>
+      </x:c>
+      <x:c r="C8" s="66" t="str">
+        <x:v>Never show terminated/paid/running without remote/PSP confirmation; recovery from outage/crash</x:v>
+      </x:c>
+      <x:c r="D8" s="66" t="str">
+        <x:v>Forced-failure integration tests; dead-letter alert evidence</x:v>
+      </x:c>
+      <x:c r="E8" s="66" t="str">
+        <x:v>Provisioning, billing, UX</x:v>
+      </x:c>
+      <x:c r="F8" s="66" t="str">
+        <x:v>BLOCKED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="64" customHeight="1">
+      <x:c r="A9" s="66" t="str">
+        <x:v>05</x:v>
+      </x:c>
+      <x:c r="B9" s="66" t="str">
+        <x:v>Operational readiness</x:v>
+      </x:c>
+      <x:c r="C9" s="66" t="str">
+        <x:v>Backup/restore test, secret rotation plan, mail deliverability, structured alerts, rate-limit, TLS headers</x:v>
+      </x:c>
+      <x:c r="D9" s="66" t="str">
+        <x:v>Documented restore drill + security test results</x:v>
+      </x:c>
+      <x:c r="E9" s="66" t="str">
+        <x:v>Operations</x:v>
+      </x:c>
+      <x:c r="F9" s="66" t="str">
+        <x:v>UNVERIFIED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="64" customHeight="1">
+      <x:c r="A10" s="66" t="str">
+        <x:v>06</x:v>
+      </x:c>
+      <x:c r="B10" s="66" t="str">
+        <x:v>Smart Petal interaction QA</x:v>
+      </x:c>
+      <x:c r="C10" s="66" t="str">
+        <x:v>One canonical tab/navigation/status model, no dead Manage buttons, responsive, safe loading/error and action permissions</x:v>
+      </x:c>
+      <x:c r="D10" s="66" t="str">
+        <x:v>Screenshots against Fortless Views; role/provider/status matrix</x:v>
+      </x:c>
+      <x:c r="E10" s="66" t="str">
+        <x:v>UI/UX</x:v>
+      </x:c>
+      <x:c r="F10" s="66" t="str">
+        <x:v>UNVERIFIED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="64" customHeight="1">
+      <x:c r="A11" s="66" t="str">
+        <x:v>07</x:v>
+      </x:c>
+      <x:c r="B11" s="66" t="str">
+        <x:v>Controlled launch</x:v>
+      </x:c>
+      <x:c r="C11" s="66" t="str">
+        <x:v>Start with internal test account then small invite-only paid pilot, manual support and rollback procedure</x:v>
+      </x:c>
+      <x:c r="D11" s="66" t="str">
+        <x:v>Signed go/no-go checklist + incident owner + pilot feedback</x:v>
+      </x:c>
+      <x:c r="E11" s="66" t="str">
+        <x:v>Business operations</x:v>
+      </x:c>
+      <x:c r="F11" s="66" t="str">
+        <x:v>NOT STARTED</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:F1"/>
+    <x:mergeCell ref="A2:F2"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>